<commit_message>
Decode column encodings in all thirteen readers, and measure what they bought
The writer picked encodings already; now every generated reader decodes them.
Each language gained a column cursor - the one place that knows how a delta
accumulates, how long a run has left, and that a dictionary index is a reference
into strings decoded once - while its row loop stays a row loop.

The conformance corpus grew rows shaped so that all seven encodings win
somewhere, and a test pins which column each one wins, so the coverage cannot
narrow quietly.

Measured on the rescue dataset: 7.84 MB to 0.36 MB, load 24 ms to 8 ms, and
resident memory 27.6 MB to 11.9 MB - the last because a column of three distinct
strings now allocates three, not 103,395. The docs are rewritten around the new
numbers, and spec/ gains the rationale for the column-oriented layout itself.
</commit_message>
<xml_diff>
--- a/test/fixtures/xlsx/conformance/conformance.xlsx
+++ b/test/fixtures/xlsx/conformance/conformance.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="251">
   <si>
     <t xml:space="preserve">~~enum:Flag~~</t>
   </si>
@@ -401,6 +401,249 @@
     <t xml:space="preserve">é</t>
   </si>
   <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741829</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741831</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741840</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741843</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741850</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741851</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741859</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741863</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741869</t>
+  </si>
+  <si>
+    <t xml:space="preserve">24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741871</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741876</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">beta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741878</t>
+  </si>
+  <si>
+    <t xml:space="preserve">33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741887</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741890</t>
+  </si>
+  <si>
+    <t xml:space="preserve">39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741897</t>
+  </si>
+  <si>
+    <t xml:space="preserve">42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741898</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741906</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741910</t>
+  </si>
+  <si>
+    <t xml:space="preserve">51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741916</t>
+  </si>
+  <si>
+    <t xml:space="preserve">54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741918</t>
+  </si>
+  <si>
+    <t xml:space="preserve">57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741923</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gamma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741925</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741934</t>
+  </si>
+  <si>
+    <t xml:space="preserve">66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741937</t>
+  </si>
+  <si>
+    <t xml:space="preserve">69</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741944</t>
+  </si>
+  <si>
+    <t xml:space="preserve">72</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741945</t>
+  </si>
+  <si>
+    <t xml:space="preserve">75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741953</t>
+  </si>
+  <si>
+    <t xml:space="preserve">78</t>
+  </si>
+  <si>
+    <t xml:space="preserve">34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741957</t>
+  </si>
+  <si>
+    <t xml:space="preserve">81</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741963</t>
+  </si>
+  <si>
+    <t xml:space="preserve">84</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1073741965</t>
+  </si>
+  <si>
+    <t xml:space="preserve">87</t>
+  </si>
+  <si>
     <t xml:space="preserve">~~table:Owners~~</t>
   </si>
   <si>
@@ -419,19 +662,49 @@
     <t xml:space="preserve">first</t>
   </si>
   <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
     <t xml:space="preserve">second</t>
   </si>
   <si>
-    <t xml:space="preserve">20</t>
-  </si>
-  <si>
     <t xml:space="preserve">third</t>
   </si>
   <si>
-    <t xml:space="preserve">30</t>
+    <t xml:space="preserve">red</t>
+  </si>
+  <si>
+    <t xml:space="preserve">40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">blue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">70</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">90</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">110</t>
+  </si>
+  <si>
+    <t xml:space="preserve">120</t>
+  </si>
+  <si>
+    <t xml:space="preserve">130</t>
+  </si>
+  <si>
+    <t xml:space="preserve">140</t>
+  </si>
+  <si>
+    <t xml:space="preserve">150</t>
   </si>
   <si>
     <t xml:space="preserve">~~const:Limits~~</t>
@@ -456,9 +729,6 @@
   </si>
   <si>
     <t xml:space="preserve">Ratio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.25</t>
   </si>
   <si>
     <t xml:space="preserve">Precise</t>
@@ -539,7 +809,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="B2:Y33"/>
+  <dimension ref="B2:Y68"/>
   <sheetFormatPr defaultColWidth="8.43" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -1186,20 +1456,434 @@
         <v>9</v>
       </c>
     </row>
+    <row r="15">
+      <c r="I15" t="s">
+        <v>129</v>
+      </c>
+      <c r="J15" t="s">
+        <v>130</v>
+      </c>
+      <c r="K15" t="s">
+        <v>6</v>
+      </c>
+      <c r="L15" t="s">
+        <v>131</v>
+      </c>
+      <c r="M15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N15" t="s">
+        <v>133</v>
+      </c>
+      <c r="O15" t="s">
+        <v>81</v>
+      </c>
+      <c r="P15" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>83</v>
+      </c>
+      <c r="R15" t="s">
+        <v>84</v>
+      </c>
+      <c r="S15" t="s">
+        <v>8</v>
+      </c>
+      <c r="T15" t="s">
+        <v>22</v>
+      </c>
+      <c r="U15" t="s">
+        <v>22</v>
+      </c>
+      <c r="V15" t="s">
+        <v>22</v>
+      </c>
+      <c r="W15" t="s">
+        <v>22</v>
+      </c>
+      <c r="X15" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y15" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="I16" t="s">
+        <v>134</v>
+      </c>
+      <c r="J16" t="s">
+        <v>135</v>
+      </c>
+      <c r="K16" t="s">
+        <v>87</v>
+      </c>
+      <c r="L16" t="s">
+        <v>131</v>
+      </c>
+      <c r="M16" t="s">
+        <v>132</v>
+      </c>
+      <c r="N16" t="s">
+        <v>133</v>
+      </c>
+      <c r="O16" t="s">
+        <v>72</v>
+      </c>
+      <c r="P16" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>83</v>
+      </c>
+      <c r="R16" t="s">
+        <v>84</v>
+      </c>
+      <c r="S16" t="s">
+        <v>8</v>
+      </c>
+      <c r="T16" t="s">
+        <v>22</v>
+      </c>
+      <c r="U16" t="s">
+        <v>22</v>
+      </c>
+      <c r="V16" t="s">
+        <v>22</v>
+      </c>
+      <c r="W16" t="s">
+        <v>22</v>
+      </c>
+      <c r="X16" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y16" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="I17" t="s">
+        <v>136</v>
+      </c>
+      <c r="J17" t="s">
+        <v>137</v>
+      </c>
+      <c r="K17" t="s">
+        <v>119</v>
+      </c>
+      <c r="L17" t="s">
+        <v>131</v>
+      </c>
+      <c r="M17" t="s">
+        <v>132</v>
+      </c>
+      <c r="N17" t="s">
+        <v>133</v>
+      </c>
+      <c r="O17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P17" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>83</v>
+      </c>
+      <c r="R17" t="s">
+        <v>84</v>
+      </c>
+      <c r="S17" t="s">
+        <v>8</v>
+      </c>
+      <c r="T17" t="s">
+        <v>22</v>
+      </c>
+      <c r="U17" t="s">
+        <v>22</v>
+      </c>
+      <c r="V17" t="s">
+        <v>22</v>
+      </c>
+      <c r="W17" t="s">
+        <v>22</v>
+      </c>
+      <c r="X17" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="I18" t="s">
+        <v>138</v>
+      </c>
+      <c r="J18" t="s">
+        <v>139</v>
+      </c>
+      <c r="K18" t="s">
+        <v>136</v>
+      </c>
+      <c r="L18" t="s">
+        <v>131</v>
+      </c>
+      <c r="M18" t="s">
+        <v>132</v>
+      </c>
+      <c r="N18" t="s">
+        <v>133</v>
+      </c>
+      <c r="O18" t="s">
+        <v>72</v>
+      </c>
+      <c r="P18" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>83</v>
+      </c>
+      <c r="R18" t="s">
+        <v>84</v>
+      </c>
+      <c r="S18" t="s">
+        <v>8</v>
+      </c>
+      <c r="T18" t="s">
+        <v>22</v>
+      </c>
+      <c r="U18" t="s">
+        <v>22</v>
+      </c>
+      <c r="V18" t="s">
+        <v>22</v>
+      </c>
+      <c r="W18" t="s">
+        <v>22</v>
+      </c>
+      <c r="X18" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="I19" t="s">
+        <v>140</v>
+      </c>
+      <c r="J19" t="s">
+        <v>141</v>
+      </c>
+      <c r="K19" t="s">
+        <v>142</v>
+      </c>
+      <c r="L19" t="s">
+        <v>131</v>
+      </c>
+      <c r="M19" t="s">
+        <v>132</v>
+      </c>
+      <c r="N19" t="s">
+        <v>133</v>
+      </c>
+      <c r="O19" t="s">
+        <v>81</v>
+      </c>
+      <c r="P19" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>83</v>
+      </c>
+      <c r="R19" t="s">
+        <v>84</v>
+      </c>
+      <c r="S19" t="s">
+        <v>8</v>
+      </c>
+      <c r="T19" t="s">
+        <v>22</v>
+      </c>
+      <c r="U19" t="s">
+        <v>22</v>
+      </c>
+      <c r="V19" t="s">
+        <v>22</v>
+      </c>
+      <c r="W19" t="s">
+        <v>22</v>
+      </c>
+      <c r="X19" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="I20" t="s">
+        <v>142</v>
+      </c>
+      <c r="J20" t="s">
+        <v>143</v>
+      </c>
+      <c r="K20" t="s">
+        <v>144</v>
+      </c>
+      <c r="L20" t="s">
+        <v>131</v>
+      </c>
+      <c r="M20" t="s">
+        <v>132</v>
+      </c>
+      <c r="N20" t="s">
+        <v>133</v>
+      </c>
+      <c r="O20" t="s">
+        <v>72</v>
+      </c>
+      <c r="P20" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>83</v>
+      </c>
+      <c r="R20" t="s">
+        <v>84</v>
+      </c>
+      <c r="S20" t="s">
+        <v>8</v>
+      </c>
+      <c r="T20" t="s">
+        <v>22</v>
+      </c>
+      <c r="U20" t="s">
+        <v>22</v>
+      </c>
+      <c r="V20" t="s">
+        <v>22</v>
+      </c>
+      <c r="W20" t="s">
+        <v>22</v>
+      </c>
+      <c r="X20" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>76</v>
+      </c>
+    </row>
     <row r="21">
       <c r="B21" t="s">
-        <v>140</v>
+        <v>231</v>
       </c>
       <c r="I21" t="s">
-        <v>129</v>
+        <v>145</v>
+      </c>
+      <c r="J21" t="s">
+        <v>146</v>
+      </c>
+      <c r="K21" t="s">
+        <v>147</v>
+      </c>
+      <c r="L21" t="s">
+        <v>131</v>
+      </c>
+      <c r="M21" t="s">
+        <v>132</v>
+      </c>
+      <c r="N21" t="s">
+        <v>133</v>
+      </c>
+      <c r="O21" t="s">
+        <v>81</v>
+      </c>
+      <c r="P21" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>83</v>
+      </c>
+      <c r="R21" t="s">
+        <v>84</v>
+      </c>
+      <c r="S21" t="s">
+        <v>8</v>
+      </c>
+      <c r="T21" t="s">
+        <v>22</v>
+      </c>
+      <c r="U21" t="s">
+        <v>22</v>
+      </c>
+      <c r="V21" t="s">
+        <v>22</v>
+      </c>
+      <c r="W21" t="s">
+        <v>22</v>
+      </c>
+      <c r="X21" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s">
-        <v>141</v>
+        <v>232</v>
       </c>
       <c r="I22" t="s">
-        <v>130</v>
+        <v>148</v>
+      </c>
+      <c r="J22" t="s">
+        <v>149</v>
+      </c>
+      <c r="K22" t="s">
+        <v>150</v>
+      </c>
+      <c r="L22" t="s">
+        <v>131</v>
+      </c>
+      <c r="M22" t="s">
+        <v>132</v>
+      </c>
+      <c r="N22" t="s">
+        <v>133</v>
+      </c>
+      <c r="O22" t="s">
+        <v>72</v>
+      </c>
+      <c r="P22" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>83</v>
+      </c>
+      <c r="R22" t="s">
+        <v>84</v>
+      </c>
+      <c r="S22" t="s">
+        <v>8</v>
+      </c>
+      <c r="T22" t="s">
+        <v>22</v>
+      </c>
+      <c r="U22" t="s">
+        <v>22</v>
+      </c>
+      <c r="V22" t="s">
+        <v>22</v>
+      </c>
+      <c r="W22" t="s">
+        <v>22</v>
+      </c>
+      <c r="X22" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y22" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="23">
@@ -1207,10 +1891,10 @@
         <v>2</v>
       </c>
       <c r="C23" t="s">
-        <v>142</v>
+        <v>233</v>
       </c>
       <c r="D23" t="s">
-        <v>143</v>
+        <v>234</v>
       </c>
       <c r="E23" t="s">
         <v>3</v>
@@ -1219,18 +1903,60 @@
         <v>4</v>
       </c>
       <c r="I23" t="s">
-        <v>19</v>
+        <v>144</v>
       </c>
       <c r="J23" t="s">
-        <v>2</v>
+        <v>151</v>
       </c>
       <c r="K23" t="s">
+        <v>152</v>
+      </c>
+      <c r="L23" t="s">
+        <v>131</v>
+      </c>
+      <c r="M23" t="s">
         <v>132</v>
+      </c>
+      <c r="N23" t="s">
+        <v>133</v>
+      </c>
+      <c r="O23" t="s">
+        <v>81</v>
+      </c>
+      <c r="P23" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>83</v>
+      </c>
+      <c r="R23" t="s">
+        <v>84</v>
+      </c>
+      <c r="S23" t="s">
+        <v>8</v>
+      </c>
+      <c r="T23" t="s">
+        <v>22</v>
+      </c>
+      <c r="U23" t="s">
+        <v>22</v>
+      </c>
+      <c r="V23" t="s">
+        <v>22</v>
+      </c>
+      <c r="W23" t="s">
+        <v>22</v>
+      </c>
+      <c r="X23" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y23" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s">
-        <v>144</v>
+        <v>235</v>
       </c>
       <c r="C24" t="s">
         <v>21</v>
@@ -1239,24 +1965,66 @@
         <v>22</v>
       </c>
       <c r="E24" t="s">
+        <v>144</v>
+      </c>
+      <c r="F24" t="s">
+        <v>236</v>
+      </c>
+      <c r="I24" t="s">
+        <v>153</v>
+      </c>
+      <c r="J24" t="s">
+        <v>154</v>
+      </c>
+      <c r="K24" t="s">
+        <v>155</v>
+      </c>
+      <c r="L24" t="s">
+        <v>131</v>
+      </c>
+      <c r="M24" t="s">
+        <v>132</v>
+      </c>
+      <c r="N24" t="s">
+        <v>133</v>
+      </c>
+      <c r="O24" t="s">
+        <v>72</v>
+      </c>
+      <c r="P24" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>83</v>
+      </c>
+      <c r="R24" t="s">
+        <v>84</v>
+      </c>
+      <c r="S24" t="s">
+        <v>8</v>
+      </c>
+      <c r="T24" t="s">
+        <v>22</v>
+      </c>
+      <c r="U24" t="s">
+        <v>22</v>
+      </c>
+      <c r="V24" t="s">
+        <v>22</v>
+      </c>
+      <c r="W24" t="s">
+        <v>22</v>
+      </c>
+      <c r="X24" t="s">
         <v>87</v>
       </c>
-      <c r="F24" t="s">
-        <v>145</v>
-      </c>
-      <c r="I24" t="s">
-        <v>20</v>
-      </c>
-      <c r="J24" t="s">
-        <v>131</v>
-      </c>
-      <c r="K24" t="s">
-        <v>133</v>
+      <c r="Y24" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="s">
-        <v>146</v>
+        <v>237</v>
       </c>
       <c r="C25" t="s">
         <v>28</v>
@@ -1271,18 +2039,60 @@
         <v>27</v>
       </c>
       <c r="I25" t="s">
-        <v>21</v>
+        <v>156</v>
       </c>
       <c r="J25" t="s">
-        <v>37</v>
+        <v>157</v>
       </c>
       <c r="K25" t="s">
-        <v>21</v>
+        <v>158</v>
+      </c>
+      <c r="L25" t="s">
+        <v>131</v>
+      </c>
+      <c r="M25" t="s">
+        <v>132</v>
+      </c>
+      <c r="N25" t="s">
+        <v>159</v>
+      </c>
+      <c r="O25" t="s">
+        <v>81</v>
+      </c>
+      <c r="P25" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>83</v>
+      </c>
+      <c r="R25" t="s">
+        <v>84</v>
+      </c>
+      <c r="S25" t="s">
+        <v>8</v>
+      </c>
+      <c r="T25" t="s">
+        <v>22</v>
+      </c>
+      <c r="U25" t="s">
+        <v>22</v>
+      </c>
+      <c r="V25" t="s">
+        <v>22</v>
+      </c>
+      <c r="W25" t="s">
+        <v>22</v>
+      </c>
+      <c r="X25" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y25" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="s">
-        <v>147</v>
+        <v>238</v>
       </c>
       <c r="C26" t="s">
         <v>31</v>
@@ -1291,24 +2101,66 @@
         <v>22</v>
       </c>
       <c r="E26" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="F26" t="s">
         <v>30</v>
       </c>
       <c r="I26" t="s">
-        <v>22</v>
+        <v>147</v>
       </c>
       <c r="J26" t="s">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="K26" t="s">
-        <v>22</v>
+        <v>161</v>
+      </c>
+      <c r="L26" t="s">
+        <v>131</v>
+      </c>
+      <c r="M26" t="s">
+        <v>132</v>
+      </c>
+      <c r="N26" t="s">
+        <v>159</v>
+      </c>
+      <c r="O26" t="s">
+        <v>72</v>
+      </c>
+      <c r="P26" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>83</v>
+      </c>
+      <c r="R26" t="s">
+        <v>84</v>
+      </c>
+      <c r="S26" t="s">
+        <v>8</v>
+      </c>
+      <c r="T26" t="s">
+        <v>22</v>
+      </c>
+      <c r="U26" t="s">
+        <v>22</v>
+      </c>
+      <c r="V26" t="s">
+        <v>22</v>
+      </c>
+      <c r="W26" t="s">
+        <v>22</v>
+      </c>
+      <c r="X26" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y26" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="s">
-        <v>149</v>
+        <v>239</v>
       </c>
       <c r="C27" t="s">
         <v>34</v>
@@ -1320,21 +2172,63 @@
         <v>112</v>
       </c>
       <c r="F27" t="s">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="I27" t="s">
-        <v>23</v>
+        <v>162</v>
       </c>
       <c r="J27" t="s">
-        <v>23</v>
+        <v>163</v>
       </c>
       <c r="K27" t="s">
-        <v>23</v>
+        <v>164</v>
+      </c>
+      <c r="L27" t="s">
+        <v>131</v>
+      </c>
+      <c r="M27" t="s">
+        <v>132</v>
+      </c>
+      <c r="N27" t="s">
+        <v>159</v>
+      </c>
+      <c r="O27" t="s">
+        <v>81</v>
+      </c>
+      <c r="P27" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>83</v>
+      </c>
+      <c r="R27" t="s">
+        <v>84</v>
+      </c>
+      <c r="S27" t="s">
+        <v>8</v>
+      </c>
+      <c r="T27" t="s">
+        <v>22</v>
+      </c>
+      <c r="U27" t="s">
+        <v>22</v>
+      </c>
+      <c r="V27" t="s">
+        <v>22</v>
+      </c>
+      <c r="W27" t="s">
+        <v>22</v>
+      </c>
+      <c r="X27" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y27" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" t="s">
-        <v>151</v>
+        <v>241</v>
       </c>
       <c r="C28" t="s">
         <v>37</v>
@@ -1346,21 +2240,63 @@
         <v>91</v>
       </c>
       <c r="F28" t="s">
-        <v>152</v>
+        <v>242</v>
       </c>
       <c r="I28" t="s">
+        <v>165</v>
+      </c>
+      <c r="J28" t="s">
+        <v>166</v>
+      </c>
+      <c r="K28" t="s">
+        <v>167</v>
+      </c>
+      <c r="L28" t="s">
+        <v>131</v>
+      </c>
+      <c r="M28" t="s">
+        <v>132</v>
+      </c>
+      <c r="N28" t="s">
+        <v>159</v>
+      </c>
+      <c r="O28" t="s">
+        <v>72</v>
+      </c>
+      <c r="P28" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>83</v>
+      </c>
+      <c r="R28" t="s">
+        <v>84</v>
+      </c>
+      <c r="S28" t="s">
+        <v>8</v>
+      </c>
+      <c r="T28" t="s">
+        <v>22</v>
+      </c>
+      <c r="U28" t="s">
+        <v>22</v>
+      </c>
+      <c r="V28" t="s">
+        <v>22</v>
+      </c>
+      <c r="W28" t="s">
+        <v>22</v>
+      </c>
+      <c r="X28" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y28" t="s">
         <v>9</v>
-      </c>
-      <c r="J28" t="s">
-        <v>134</v>
-      </c>
-      <c r="K28" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="s">
-        <v>153</v>
+        <v>243</v>
       </c>
       <c r="C29" t="s">
         <v>40</v>
@@ -1372,21 +2308,63 @@
         <v>81</v>
       </c>
       <c r="F29" t="s">
-        <v>154</v>
+        <v>244</v>
       </c>
       <c r="I29" t="s">
+        <v>150</v>
+      </c>
+      <c r="J29" t="s">
+        <v>168</v>
+      </c>
+      <c r="K29" t="s">
+        <v>169</v>
+      </c>
+      <c r="L29" t="s">
+        <v>131</v>
+      </c>
+      <c r="M29" t="s">
+        <v>132</v>
+      </c>
+      <c r="N29" t="s">
+        <v>159</v>
+      </c>
+      <c r="O29" t="s">
+        <v>81</v>
+      </c>
+      <c r="P29" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q29" t="s">
+        <v>83</v>
+      </c>
+      <c r="R29" t="s">
+        <v>84</v>
+      </c>
+      <c r="S29" t="s">
+        <v>8</v>
+      </c>
+      <c r="T29" t="s">
+        <v>22</v>
+      </c>
+      <c r="U29" t="s">
+        <v>22</v>
+      </c>
+      <c r="V29" t="s">
+        <v>22</v>
+      </c>
+      <c r="W29" t="s">
+        <v>22</v>
+      </c>
+      <c r="X29" t="s">
         <v>76</v>
       </c>
-      <c r="J29" t="s">
-        <v>136</v>
-      </c>
-      <c r="K29" t="s">
-        <v>137</v>
+      <c r="Y29" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="s">
-        <v>155</v>
+        <v>245</v>
       </c>
       <c r="C30" t="s">
         <v>43</v>
@@ -1401,18 +2379,60 @@
         <v>42</v>
       </c>
       <c r="I30" t="s">
+        <v>170</v>
+      </c>
+      <c r="J30" t="s">
+        <v>171</v>
+      </c>
+      <c r="K30" t="s">
+        <v>172</v>
+      </c>
+      <c r="L30" t="s">
+        <v>131</v>
+      </c>
+      <c r="M30" t="s">
+        <v>132</v>
+      </c>
+      <c r="N30" t="s">
+        <v>159</v>
+      </c>
+      <c r="O30" t="s">
+        <v>72</v>
+      </c>
+      <c r="P30" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>83</v>
+      </c>
+      <c r="R30" t="s">
+        <v>84</v>
+      </c>
+      <c r="S30" t="s">
+        <v>11</v>
+      </c>
+      <c r="T30" t="s">
+        <v>22</v>
+      </c>
+      <c r="U30" t="s">
+        <v>22</v>
+      </c>
+      <c r="V30" t="s">
+        <v>22</v>
+      </c>
+      <c r="W30" t="s">
+        <v>22</v>
+      </c>
+      <c r="X30" t="s">
         <v>87</v>
       </c>
-      <c r="J30" t="s">
-        <v>138</v>
-      </c>
-      <c r="K30" t="s">
-        <v>139</v>
+      <c r="Y30" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="31">
       <c r="B31" t="s">
-        <v>156</v>
+        <v>246</v>
       </c>
       <c r="C31" t="s">
         <v>45</v>
@@ -1426,10 +2446,61 @@
       <c r="F31" t="s">
         <v>42</v>
       </c>
+      <c r="I31" t="s">
+        <v>173</v>
+      </c>
+      <c r="J31" t="s">
+        <v>174</v>
+      </c>
+      <c r="K31" t="s">
+        <v>175</v>
+      </c>
+      <c r="L31" t="s">
+        <v>131</v>
+      </c>
+      <c r="M31" t="s">
+        <v>132</v>
+      </c>
+      <c r="N31" t="s">
+        <v>159</v>
+      </c>
+      <c r="O31" t="s">
+        <v>81</v>
+      </c>
+      <c r="P31" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>83</v>
+      </c>
+      <c r="R31" t="s">
+        <v>84</v>
+      </c>
+      <c r="S31" t="s">
+        <v>11</v>
+      </c>
+      <c r="T31" t="s">
+        <v>22</v>
+      </c>
+      <c r="U31" t="s">
+        <v>22</v>
+      </c>
+      <c r="V31" t="s">
+        <v>22</v>
+      </c>
+      <c r="W31" t="s">
+        <v>22</v>
+      </c>
+      <c r="X31" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" t="s">
-        <v>157</v>
+        <v>247</v>
       </c>
       <c r="C32" t="s">
         <v>51</v>
@@ -1441,12 +2512,63 @@
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>158</v>
+        <v>248</v>
+      </c>
+      <c r="I32" t="s">
+        <v>152</v>
+      </c>
+      <c r="J32" t="s">
+        <v>176</v>
+      </c>
+      <c r="K32" t="s">
+        <v>177</v>
+      </c>
+      <c r="L32" t="s">
+        <v>131</v>
+      </c>
+      <c r="M32" t="s">
+        <v>132</v>
+      </c>
+      <c r="N32" t="s">
+        <v>159</v>
+      </c>
+      <c r="O32" t="s">
+        <v>72</v>
+      </c>
+      <c r="P32" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>83</v>
+      </c>
+      <c r="R32" t="s">
+        <v>84</v>
+      </c>
+      <c r="S32" t="s">
+        <v>11</v>
+      </c>
+      <c r="T32" t="s">
+        <v>22</v>
+      </c>
+      <c r="U32" t="s">
+        <v>22</v>
+      </c>
+      <c r="V32" t="s">
+        <v>22</v>
+      </c>
+      <c r="W32" t="s">
+        <v>22</v>
+      </c>
+      <c r="X32" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y32" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" t="s">
-        <v>159</v>
+        <v>249</v>
       </c>
       <c r="C33" t="s">
         <v>48</v>
@@ -1458,7 +2580,871 @@
         <v>84</v>
       </c>
       <c r="F33" t="s">
-        <v>160</v>
+        <v>250</v>
+      </c>
+      <c r="I33" t="s">
+        <v>178</v>
+      </c>
+      <c r="J33" t="s">
+        <v>179</v>
+      </c>
+      <c r="K33" t="s">
+        <v>180</v>
+      </c>
+      <c r="L33" t="s">
+        <v>131</v>
+      </c>
+      <c r="M33" t="s">
+        <v>132</v>
+      </c>
+      <c r="N33" t="s">
+        <v>159</v>
+      </c>
+      <c r="O33" t="s">
+        <v>81</v>
+      </c>
+      <c r="P33" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>83</v>
+      </c>
+      <c r="R33" t="s">
+        <v>84</v>
+      </c>
+      <c r="S33" t="s">
+        <v>11</v>
+      </c>
+      <c r="T33" t="s">
+        <v>22</v>
+      </c>
+      <c r="U33" t="s">
+        <v>22</v>
+      </c>
+      <c r="V33" t="s">
+        <v>22</v>
+      </c>
+      <c r="W33" t="s">
+        <v>22</v>
+      </c>
+      <c r="X33" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="I34" t="s">
+        <v>181</v>
+      </c>
+      <c r="J34" t="s">
+        <v>182</v>
+      </c>
+      <c r="K34" t="s">
+        <v>183</v>
+      </c>
+      <c r="L34" t="s">
+        <v>131</v>
+      </c>
+      <c r="M34" t="s">
+        <v>132</v>
+      </c>
+      <c r="N34" t="s">
+        <v>159</v>
+      </c>
+      <c r="O34" t="s">
+        <v>72</v>
+      </c>
+      <c r="P34" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>83</v>
+      </c>
+      <c r="R34" t="s">
+        <v>84</v>
+      </c>
+      <c r="S34" t="s">
+        <v>11</v>
+      </c>
+      <c r="T34" t="s">
+        <v>22</v>
+      </c>
+      <c r="U34" t="s">
+        <v>22</v>
+      </c>
+      <c r="V34" t="s">
+        <v>22</v>
+      </c>
+      <c r="W34" t="s">
+        <v>22</v>
+      </c>
+      <c r="X34" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="I35" t="s">
+        <v>155</v>
+      </c>
+      <c r="J35" t="s">
+        <v>184</v>
+      </c>
+      <c r="K35" t="s">
+        <v>185</v>
+      </c>
+      <c r="L35" t="s">
+        <v>131</v>
+      </c>
+      <c r="M35" t="s">
+        <v>132</v>
+      </c>
+      <c r="N35" t="s">
+        <v>186</v>
+      </c>
+      <c r="O35" t="s">
+        <v>81</v>
+      </c>
+      <c r="P35" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>83</v>
+      </c>
+      <c r="R35" t="s">
+        <v>84</v>
+      </c>
+      <c r="S35" t="s">
+        <v>11</v>
+      </c>
+      <c r="T35" t="s">
+        <v>22</v>
+      </c>
+      <c r="U35" t="s">
+        <v>22</v>
+      </c>
+      <c r="V35" t="s">
+        <v>22</v>
+      </c>
+      <c r="W35" t="s">
+        <v>22</v>
+      </c>
+      <c r="X35" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="I36" t="s">
+        <v>187</v>
+      </c>
+      <c r="J36" t="s">
+        <v>188</v>
+      </c>
+      <c r="K36" t="s">
+        <v>77</v>
+      </c>
+      <c r="L36" t="s">
+        <v>131</v>
+      </c>
+      <c r="M36" t="s">
+        <v>132</v>
+      </c>
+      <c r="N36" t="s">
+        <v>186</v>
+      </c>
+      <c r="O36" t="s">
+        <v>72</v>
+      </c>
+      <c r="P36" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>83</v>
+      </c>
+      <c r="R36" t="s">
+        <v>84</v>
+      </c>
+      <c r="S36" t="s">
+        <v>11</v>
+      </c>
+      <c r="T36" t="s">
+        <v>22</v>
+      </c>
+      <c r="U36" t="s">
+        <v>22</v>
+      </c>
+      <c r="V36" t="s">
+        <v>22</v>
+      </c>
+      <c r="W36" t="s">
+        <v>22</v>
+      </c>
+      <c r="X36" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="I37" t="s">
+        <v>189</v>
+      </c>
+      <c r="J37" t="s">
+        <v>190</v>
+      </c>
+      <c r="K37" t="s">
+        <v>191</v>
+      </c>
+      <c r="L37" t="s">
+        <v>131</v>
+      </c>
+      <c r="M37" t="s">
+        <v>132</v>
+      </c>
+      <c r="N37" t="s">
+        <v>186</v>
+      </c>
+      <c r="O37" t="s">
+        <v>81</v>
+      </c>
+      <c r="P37" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>83</v>
+      </c>
+      <c r="R37" t="s">
+        <v>84</v>
+      </c>
+      <c r="S37" t="s">
+        <v>11</v>
+      </c>
+      <c r="T37" t="s">
+        <v>22</v>
+      </c>
+      <c r="U37" t="s">
+        <v>22</v>
+      </c>
+      <c r="V37" t="s">
+        <v>22</v>
+      </c>
+      <c r="W37" t="s">
+        <v>22</v>
+      </c>
+      <c r="X37" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y37" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="I38" t="s">
+        <v>158</v>
+      </c>
+      <c r="J38" t="s">
+        <v>192</v>
+      </c>
+      <c r="K38" t="s">
+        <v>193</v>
+      </c>
+      <c r="L38" t="s">
+        <v>131</v>
+      </c>
+      <c r="M38" t="s">
+        <v>132</v>
+      </c>
+      <c r="N38" t="s">
+        <v>186</v>
+      </c>
+      <c r="O38" t="s">
+        <v>72</v>
+      </c>
+      <c r="P38" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>83</v>
+      </c>
+      <c r="R38" t="s">
+        <v>84</v>
+      </c>
+      <c r="S38" t="s">
+        <v>11</v>
+      </c>
+      <c r="T38" t="s">
+        <v>22</v>
+      </c>
+      <c r="U38" t="s">
+        <v>22</v>
+      </c>
+      <c r="V38" t="s">
+        <v>22</v>
+      </c>
+      <c r="W38" t="s">
+        <v>22</v>
+      </c>
+      <c r="X38" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y38" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="I39" t="s">
+        <v>194</v>
+      </c>
+      <c r="J39" t="s">
+        <v>195</v>
+      </c>
+      <c r="K39" t="s">
+        <v>196</v>
+      </c>
+      <c r="L39" t="s">
+        <v>131</v>
+      </c>
+      <c r="M39" t="s">
+        <v>132</v>
+      </c>
+      <c r="N39" t="s">
+        <v>186</v>
+      </c>
+      <c r="O39" t="s">
+        <v>81</v>
+      </c>
+      <c r="P39" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>83</v>
+      </c>
+      <c r="R39" t="s">
+        <v>84</v>
+      </c>
+      <c r="S39" t="s">
+        <v>11</v>
+      </c>
+      <c r="T39" t="s">
+        <v>22</v>
+      </c>
+      <c r="U39" t="s">
+        <v>22</v>
+      </c>
+      <c r="V39" t="s">
+        <v>22</v>
+      </c>
+      <c r="W39" t="s">
+        <v>22</v>
+      </c>
+      <c r="X39" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y39" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="I40" t="s">
+        <v>197</v>
+      </c>
+      <c r="J40" t="s">
+        <v>198</v>
+      </c>
+      <c r="K40" t="s">
+        <v>199</v>
+      </c>
+      <c r="L40" t="s">
+        <v>131</v>
+      </c>
+      <c r="M40" t="s">
+        <v>132</v>
+      </c>
+      <c r="N40" t="s">
+        <v>186</v>
+      </c>
+      <c r="O40" t="s">
+        <v>72</v>
+      </c>
+      <c r="P40" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q40" t="s">
+        <v>83</v>
+      </c>
+      <c r="R40" t="s">
+        <v>84</v>
+      </c>
+      <c r="S40" t="s">
+        <v>11</v>
+      </c>
+      <c r="T40" t="s">
+        <v>22</v>
+      </c>
+      <c r="U40" t="s">
+        <v>22</v>
+      </c>
+      <c r="V40" t="s">
+        <v>22</v>
+      </c>
+      <c r="W40" t="s">
+        <v>22</v>
+      </c>
+      <c r="X40" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y40" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="I41" t="s">
+        <v>161</v>
+      </c>
+      <c r="J41" t="s">
+        <v>200</v>
+      </c>
+      <c r="K41" t="s">
+        <v>201</v>
+      </c>
+      <c r="L41" t="s">
+        <v>131</v>
+      </c>
+      <c r="M41" t="s">
+        <v>132</v>
+      </c>
+      <c r="N41" t="s">
+        <v>186</v>
+      </c>
+      <c r="O41" t="s">
+        <v>81</v>
+      </c>
+      <c r="P41" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>83</v>
+      </c>
+      <c r="R41" t="s">
+        <v>84</v>
+      </c>
+      <c r="S41" t="s">
+        <v>11</v>
+      </c>
+      <c r="T41" t="s">
+        <v>22</v>
+      </c>
+      <c r="U41" t="s">
+        <v>22</v>
+      </c>
+      <c r="V41" t="s">
+        <v>22</v>
+      </c>
+      <c r="W41" t="s">
+        <v>22</v>
+      </c>
+      <c r="X41" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y41" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="I42" t="s">
+        <v>202</v>
+      </c>
+      <c r="J42" t="s">
+        <v>203</v>
+      </c>
+      <c r="K42" t="s">
+        <v>204</v>
+      </c>
+      <c r="L42" t="s">
+        <v>131</v>
+      </c>
+      <c r="M42" t="s">
+        <v>132</v>
+      </c>
+      <c r="N42" t="s">
+        <v>186</v>
+      </c>
+      <c r="O42" t="s">
+        <v>72</v>
+      </c>
+      <c r="P42" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>83</v>
+      </c>
+      <c r="R42" t="s">
+        <v>84</v>
+      </c>
+      <c r="S42" t="s">
+        <v>11</v>
+      </c>
+      <c r="T42" t="s">
+        <v>22</v>
+      </c>
+      <c r="U42" t="s">
+        <v>22</v>
+      </c>
+      <c r="V42" t="s">
+        <v>22</v>
+      </c>
+      <c r="W42" t="s">
+        <v>22</v>
+      </c>
+      <c r="X42" t="s">
+        <v>87</v>
+      </c>
+      <c r="Y42" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="I43" t="s">
+        <v>205</v>
+      </c>
+      <c r="J43" t="s">
+        <v>206</v>
+      </c>
+      <c r="K43" t="s">
+        <v>207</v>
+      </c>
+      <c r="L43" t="s">
+        <v>131</v>
+      </c>
+      <c r="M43" t="s">
+        <v>132</v>
+      </c>
+      <c r="N43" t="s">
+        <v>186</v>
+      </c>
+      <c r="O43" t="s">
+        <v>81</v>
+      </c>
+      <c r="P43" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q43" t="s">
+        <v>83</v>
+      </c>
+      <c r="R43" t="s">
+        <v>84</v>
+      </c>
+      <c r="S43" t="s">
+        <v>11</v>
+      </c>
+      <c r="T43" t="s">
+        <v>22</v>
+      </c>
+      <c r="U43" t="s">
+        <v>22</v>
+      </c>
+      <c r="V43" t="s">
+        <v>22</v>
+      </c>
+      <c r="W43" t="s">
+        <v>22</v>
+      </c>
+      <c r="X43" t="s">
+        <v>9</v>
+      </c>
+      <c r="Y43" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="I44" t="s">
+        <v>164</v>
+      </c>
+      <c r="J44" t="s">
+        <v>208</v>
+      </c>
+      <c r="K44" t="s">
+        <v>209</v>
+      </c>
+      <c r="L44" t="s">
+        <v>131</v>
+      </c>
+      <c r="M44" t="s">
+        <v>132</v>
+      </c>
+      <c r="N44" t="s">
+        <v>186</v>
+      </c>
+      <c r="O44" t="s">
+        <v>72</v>
+      </c>
+      <c r="P44" t="s">
+        <v>82</v>
+      </c>
+      <c r="Q44" t="s">
+        <v>83</v>
+      </c>
+      <c r="R44" t="s">
+        <v>84</v>
+      </c>
+      <c r="S44" t="s">
+        <v>11</v>
+      </c>
+      <c r="T44" t="s">
+        <v>22</v>
+      </c>
+      <c r="U44" t="s">
+        <v>22</v>
+      </c>
+      <c r="V44" t="s">
+        <v>22</v>
+      </c>
+      <c r="W44" t="s">
+        <v>22</v>
+      </c>
+      <c r="X44" t="s">
+        <v>76</v>
+      </c>
+      <c r="Y44" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="I47" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="I48" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="I49" t="s">
+        <v>19</v>
+      </c>
+      <c r="J49" t="s">
+        <v>2</v>
+      </c>
+      <c r="K49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="I50" t="s">
+        <v>20</v>
+      </c>
+      <c r="J50" t="s">
+        <v>212</v>
+      </c>
+      <c r="K50" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="I51" t="s">
+        <v>21</v>
+      </c>
+      <c r="J51" t="s">
+        <v>37</v>
+      </c>
+      <c r="K51" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="I52" t="s">
+        <v>22</v>
+      </c>
+      <c r="J52" t="s">
+        <v>22</v>
+      </c>
+      <c r="K52" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="I53" t="s">
+        <v>23</v>
+      </c>
+      <c r="J53" t="s">
+        <v>23</v>
+      </c>
+      <c r="K53" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="I54" t="s">
+        <v>9</v>
+      </c>
+      <c r="J54" t="s">
+        <v>215</v>
+      </c>
+      <c r="K54" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="I55" t="s">
+        <v>76</v>
+      </c>
+      <c r="J55" t="s">
+        <v>216</v>
+      </c>
+      <c r="K55" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="I56" t="s">
+        <v>87</v>
+      </c>
+      <c r="J56" t="s">
+        <v>217</v>
+      </c>
+      <c r="K56" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="I57" t="s">
+        <v>98</v>
+      </c>
+      <c r="J57" t="s">
+        <v>218</v>
+      </c>
+      <c r="K57" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="I58" t="s">
+        <v>108</v>
+      </c>
+      <c r="J58" t="s">
+        <v>220</v>
+      </c>
+      <c r="K58" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="I59" t="s">
+        <v>119</v>
+      </c>
+      <c r="J59" t="s">
+        <v>218</v>
+      </c>
+      <c r="K59" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="I60" t="s">
+        <v>129</v>
+      </c>
+      <c r="J60" t="s">
+        <v>220</v>
+      </c>
+      <c r="K60" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="I61" t="s">
+        <v>134</v>
+      </c>
+      <c r="J61" t="s">
+        <v>218</v>
+      </c>
+      <c r="K61" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="I62" t="s">
+        <v>136</v>
+      </c>
+      <c r="J62" t="s">
+        <v>220</v>
+      </c>
+      <c r="K62" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="I63" t="s">
+        <v>138</v>
+      </c>
+      <c r="J63" t="s">
+        <v>218</v>
+      </c>
+      <c r="K63" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="I64" t="s">
+        <v>140</v>
+      </c>
+      <c r="J64" t="s">
+        <v>220</v>
+      </c>
+      <c r="K64" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="I65" t="s">
+        <v>142</v>
+      </c>
+      <c r="J65" t="s">
+        <v>218</v>
+      </c>
+      <c r="K65" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="I66" t="s">
+        <v>145</v>
+      </c>
+      <c r="J66" t="s">
+        <v>220</v>
+      </c>
+      <c r="K66" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="I67" t="s">
+        <v>148</v>
+      </c>
+      <c r="J67" t="s">
+        <v>218</v>
+      </c>
+      <c r="K67" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="I68" t="s">
+        <v>144</v>
+      </c>
+      <c r="J68" t="s">
+        <v>220</v>
+      </c>
+      <c r="K68" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>

</xml_diff>